<commit_message>
feat: 2 days to confirm an entered time; Payment due notice to the customer when both sides have confirmed; review report updated
</commit_message>
<xml_diff>
--- a/Reports/PRs-46-47-Review-Report.xlsx
+++ b/Reports/PRs-46-47-Review-Report.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>20 findings. 0 blocking for the plans themselves; 4 high items (the app cannot yet show a pending time, no app handling of the new status, the instant-booking path cannot call the quote function as written, the quote snapshot could leak the street). All are now written into the plan as a corrections section; the one that needs new work is Task 6b.</t>
+          <t>20 findings from an independent read of both plan documents. None blocks the plans. IMPORTANT: for PR #46 only the plan TEXT is corrected (a corrections section at the top of the plan). The work behind the four high items is planned, not built: Task 6b (pending time in the contract), Task 10 (app handling of awaiting-time), flow 2 (a separate path to send the quote), Task 7 (quote snapshot without the street). See the PR 46 sheet, column Status.</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1. Each side has 7 days to confirm an entered time. 2. A customer cannot edit a quote or a quoted request; changes go through the chat and the provider sends a revised quote with the same number plus _Rev.N. 3. Fix the database guard and the timer duplicate. 4. One migration instead of two. 5. Stand-in start time: document in the README and revisit later. 6. Payment is asked only when both sides have confirmed.</t>
+          <t>1. Each side has 2 days to confirm an entered time (first set to 7 days, changed to 2 the same day). 2. A customer cannot edit a quote or a quoted request; changes go through the chat and the provider sends a revised quote with the same number plus _Rev.N. 3. Fix the database guard and the timer duplicate. 4. One migration instead of two. 5. Stand-in start time: document in the README and revisit later. 6. Payment is asked only when both sides have confirmed, and the customer then gets a Payment due message (pay-by date and reminders from the existing payment rules).</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>tsc clean in domain, web and db. Domain tests 245 passed. 9 integration specs next to the changed code: 136 tests passed (booking-time-agree, request-time, quote-confirm, quote-send, timers, cron-bookings, rls-bookings, requests-quotes, bookings). Lint clean on the changed files. drizzle-kit: no schema drift. The full suites run once at the end of the stage (Task 13).</t>
+          <t>tsc clean in domain, web and db. Domain tests 245, i18n 18, mobile 313 passed. Integration specs next to the changed code passed (booking-time-agree 12, request-time 12, quote-confirm, quote-send, timers, cron-bookings, rls-bookings, requests-quotes, bookings, booking-notifications, notification-parity, push-send). Lint clean on the changed files. drizzle-kit: no schema drift. The full suites run once at the end of the stage (Task 13).</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -922,7 +922,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Kept, checked</t>
+          <t>Changed (see R3-2)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1181,6 +1181,102 @@
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>payouts spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>R3-1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Owner change: the time to confirm is 2 days, not 7.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>TIME_ANSWER_DAYS is 2. A time entered late still moves the booking deadline out so the other side has the full 2 days; a pending time not answered in 2 days falls away.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>booking-time-agree: falls away after 2 days; 2 days after a late entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>R3-2</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Owner request: when both sides have confirmed, the customer must get a Payment due message, with payment under the existing payment rules.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>The customer gets Payment due (in-app, push, email, German and English) at the moment the booking becomes awaiting-payment, whichever side confirmed last: after the other side confirms an entered time, and when the customer confirms a quote that has a time (the provider's quote counts as their confirmation). pay_by comes from payBy(); the existing payment reminders, expiry and the pay-link rules are unchanged. A quote without a time sends nothing: nothing is due yet. This replaces the earlier choice of not telling the provider/customer in one of the two cases.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>booking-time-agree (both directions); quote-confirm (with time: notice; without time: none); booking-notifications; notification-parity</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Own-3</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>The i18n catalogue test refused two push titles that were both Payment due (new notice and the reminder).</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>The new push title reads Time confirmed: payment due (German: Termin bestätigt: Zahlung fällig).</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>i18n catalogue test</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1239,38 +1335,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Task 10 / 6a</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The app cannot show or confirm a pending agreed time: the pending-time columns are staff-only and the booking contract has no field for them.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Plan corrected: new Task 6b adds pendingTime to the contract and the booking view.</t>
-        </is>
-      </c>
+          <t>Status column: Planned means written into the plan as work still to build; Documented means the plan text was corrected and nothing else is needed. Nothing marked Planned is built yet.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Planned (Task 6b)</t>
+          <t>Read first</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -1279,28 +1369,28 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Task 10 / 12</t>
+          <t>Task 10 / 6a</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>No mobile code handles the awaiting-time status; the stand-in time would show as a real appointment.</t>
+          <t>The app cannot show or confirm a pending agreed time: the pending-time columns are staff-only and the booking contract has no field for them.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Task 10 now lists booking-status, the two actions and hiding the stand-in.</t>
+          <t>Plan corrected: new Task 6b adds pendingTime to the contract and the booking view.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Planned (Task 10)</t>
+          <t>Planned (Task 6b)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1309,28 +1399,28 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Flow 2 step 6</t>
+          <t>Task 10 / 12</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Instant booking cannot call sendQuote as written (it runs as the customer).</t>
+          <t>No mobile code handles the awaiting-time status; the stand-in time would show as a real appointment.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Flow 2 needs an owner-connection variant; written into the corrections.</t>
+          <t>Task 10 now lists booking-status, the two actions and hiding the stand-in.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Planned (flow 2)</t>
+          <t>Planned (Task 10)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -1339,58 +1429,58 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Task 7</t>
+          <t>Flow 2 step 6</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The quote snapshot (draft) is readable by both parties and could leak the street.</t>
+          <t>Instant booking cannot call sendQuote as written (it runs as the customer).</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Snapshot holds postcode and city only, or the column becomes staff-only; test required.</t>
+          <t>Flow 2 needs an owner-connection variant; written into the corrections.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Planned (Task 7)</t>
+          <t>Planned (flow 2)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Tasks 3 to 5, flow 2</t>
+          <t>Task 7</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>timeIsAcceptable lives in busy.ts, not rules.ts; assertMayPropose is in rounds.ts.</t>
+          <t>The quote snapshot (draft) is readable by both parties and could leak the street.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Corrected in the corrections section.</t>
+          <t>Snapshot holds postcode and city only, or the column becomes staff-only; test required.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Documented</t>
+          <t>Planned (Task 7)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -1399,17 +1489,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Tasks 2 and 8</t>
+          <t>Tasks 3 to 5, flow 2</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Routes and contract differ from the plan (no answer route, no union body).</t>
+          <t>timeIsAcceptable lives in busy.ts, not rules.ts; assertMayPropose is in rounds.ts.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Real route list written; Task 8 reduced to the quote lists and PDF.</t>
+          <t>Corrected in the corrections section.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1420,7 +1510,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -1429,17 +1519,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Task 1 / migrations</t>
+          <t>Tasks 2 and 8</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Migration names and count in the plan do not match what was built.</t>
+          <t>Routes and contract differ from the plan (no answer route, no union body).</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Real list written (0024, 0025, 0026 after the merge).</t>
+          <t>Real route list written; Task 8 reduced to the quote lists and PDF.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1450,7 +1540,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -1459,17 +1549,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Architecture / Task 1</t>
+          <t>Task 1 / migrations</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Contradiction about where the quote number lives.</t>
+          <t>Migration names and count in the plan do not match what was built.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Number lives in quote_documents; corrections section says so.</t>
+          <t>Real list written (0024, 0025, 0026 after the merge).</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1480,7 +1570,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -1489,28 +1579,28 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Task 7</t>
+          <t>Architecture / Task 1</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Number format clashes with the invoice numbering helper (TEST- prefix, series name).</t>
+          <t>Contradiction about where the quote number lives.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Helper formatQuoteNumber with TEST- prefix; revisions add _Rev.N (owner decision 3).</t>
+          <t>Number lives in quote_documents; corrections section says so.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Planned (Task 7)</t>
+          <t>Documented</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -1519,28 +1609,28 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Task 6a</t>
+          <t>Task 7</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The plan says the provider can decline an awaiting-time booking; not possible as built.</t>
+          <t>Number format clashes with the invoice numbering helper (TEST- prefix, series name).</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Dropped: chat or let it lapse (7 days).</t>
+          <t>Helper formatQuoteNumber with TEST- prefix; revisions add _Rev.N (owner decision 3).</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Documented</t>
+          <t>Planned (Task 7)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1554,12 +1644,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Stand-in time and no-pay-button wording out of date.</t>
+          <t>The plan says the provider can decline an awaiting-time booking; not possible as built.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Stand-in documented in the README; text corrected.</t>
+          <t>Dropped: chat or let it lapse (7 days).</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1570,7 +1660,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1579,17 +1669,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Tasks 1, 2, 6, 9</t>
+          <t>Task 6a</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Notice lists disagree (two, three, four kinds).</t>
+          <t>Stand-in time and no-pay-button wording out of date.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Four kinds; Task 9 text list corrected.</t>
+          <t>Stand-in documented in the README; text corrected.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1600,7 +1690,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1609,17 +1699,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tasks 6 and 7</t>
+          <t>Tasks 1, 2, 6, 9</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>A quote can be confirmed before it has a document; ordering.</t>
+          <t>Notice lists disagree (two, three, four kinds).</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Lists must tolerate quotes without a PDF ("PDF not available").</t>
+          <t>Four kinds; Task 9 text list corrected.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1630,7 +1720,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1639,17 +1729,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Tasks 8 and 11</t>
+          <t>Tasks 6 and 7</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>List function name clashes with an existing function; a user can be both provider and customer.</t>
+          <t>A quote can be confirmed before it has a document; ordering.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Renamed listQuoteDocuments; each user gets both lists.</t>
+          <t>Lists must tolerate quotes without a PDF ("PDF not available").</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1660,26 +1750,26 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Tasks 2 and 4</t>
+          <t>Tasks 8 and 11</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>The contract does not reject a request without a time; the server does.</t>
+          <t>List function name clashes with an existing function; a user can be both provider and customer.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Wording corrected (enforced in the domain).</t>
+          <t>Renamed listQuoteDocuments; each user gets both lists.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1690,7 +1780,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1699,17 +1789,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Task 10</t>
+          <t>Tasks 2 and 4</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>The optional reason on Reject is not in the API.</t>
+          <t>The contract does not reject a request without a time; the server does.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Dropped.</t>
+          <t>Wording corrected (enforced in the domain).</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1720,7 +1810,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1734,12 +1824,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Customer Decline route not named.</t>
+          <t>The optional reason on Reject is not in the API.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Named: the existing withdraw route.</t>
+          <t>Dropped.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1750,7 +1840,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -1759,17 +1849,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Task 12</t>
+          <t>Task 10</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Removing the old accept route would break additional tasks.</t>
+          <t>Customer Decline route not named.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>The accept route stays for additional tasks.</t>
+          <t>Named: the existing withdraw route.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1780,7 +1870,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1789,17 +1879,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Flow 2</t>
+          <t>Task 12</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Existing-code description incomplete (agreed-time callers, held statuses).</t>
+          <t>Removing the old accept route would break additional tasks.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Added to the corrections.</t>
+          <t>The accept route stays for additional tasks.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1810,29 +1900,59 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Flow 2</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Existing-code description incomplete (agreed-time callers, held statuses).</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Added to the corrections.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Documented</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Task 13 / 14</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>"Fewer clicks" not measurable; request status words not mapped; print step missing.</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Tap count, status mapping and print step added to Task 13; Task 14 stays optional.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Planned (Task 13)</t>
         </is>

</xml_diff>